<commit_message>
Remove logs from version control
</commit_message>
<xml_diff>
--- a/TestData/DSAlgo_Data_Driven_Testing.xlsx
+++ b/TestData/DSAlgo_Data_Driven_Testing.xlsx
@@ -1,28 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gayat\intellij-learning\SDET229Stars\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\syeda\IdeaProjects\SDET229Stars-temp-main\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04722E78-7539-4A82-85B7-8F7CE8D33487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B8DF646-D51A-420F-8BF8-06B87BD6D399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="DS-Introduction" sheetId="2" r:id="rId2"/>
     <sheet name="Array_Try" sheetId="3" r:id="rId3"/>
     <sheet name="arrayPracticeQuestion" sheetId="4" r:id="rId4"/>
-    <sheet name="Sheet1" sheetId="7" r:id="rId5"/>
+    <sheet name="StackQueue" sheetId="7" r:id="rId5"/>
     <sheet name="LinkedList_Try" sheetId="5" r:id="rId6"/>
     <sheet name="LinkedList_Practice" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -31,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="86">
   <si>
     <t>Username</t>
   </si>
@@ -329,6 +332,18 @@
   </si>
   <si>
     <t>https://dsportalapp.herokuapp.com/tree/practice</t>
+  </si>
+  <si>
+    <t>print 'HelloQueue'</t>
+  </si>
+  <si>
+    <t>HelloQueue</t>
+  </si>
+  <si>
+    <t>print HelloQueue</t>
+  </si>
+  <si>
+    <t>NameError: name 'HelloQueue' is not defined on line 1</t>
   </si>
 </sst>
 </file>
@@ -485,7 +500,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -665,8 +680,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -781,6 +802,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -827,7 +863,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -837,6 +873,8 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="42" applyFill="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="42"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1073,16 +1111,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultColWidth="8.26953125" defaultRowHeight="14.25" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.21875" defaultRowHeight="14.25" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="23.453125" customWidth="1"/>
-    <col min="2" max="2" width="15.7265625" customWidth="1"/>
-    <col min="3" max="3" width="25.6328125" customWidth="1"/>
-    <col min="4" max="4" width="31.26953125" customWidth="1"/>
-    <col min="5" max="5" width="34.6328125" customWidth="1"/>
+    <col min="1" max="1" width="23.44140625" customWidth="1"/>
+    <col min="2" max="2" width="15.77734375" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" customWidth="1"/>
+    <col min="4" max="4" width="31.21875" customWidth="1"/>
+    <col min="5" max="5" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.5">
+    <row r="1" spans="1:5" ht="14.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1099,7 +1137,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="14.5">
+    <row r="2" spans="1:5" ht="14.4">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1113,7 +1151,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="14.5">
+    <row r="3" spans="1:5" ht="14.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1124,12 +1162,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="14.5">
+    <row r="4" spans="1:5" ht="14.4">
       <c r="E4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="14.5">
+    <row r="5" spans="1:5" ht="14.4">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1137,7 +1175,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="14.5">
+    <row r="6" spans="1:5" ht="14.4">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1148,7 +1186,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="14.5">
+    <row r="7" spans="1:5" ht="14.4">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -1167,13 +1205,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultColWidth="8.26953125" defaultRowHeight="14.25" customHeight="1"/>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultColWidth="8.21875" defaultRowHeight="14.25" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="14.453125" customWidth="1"/>
-    <col min="3" max="3" width="43.36328125" customWidth="1"/>
-    <col min="4" max="4" width="88.81640625" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" customWidth="1"/>
+    <col min="3" max="3" width="43.33203125" customWidth="1"/>
+    <col min="4" max="4" width="88.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1247,7 +1285,6 @@
         <v>12345</v>
       </c>
     </row>
-    <row r="8" spans="1:4"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D5" r:id="rId1" xr:uid="{D2FDE1DB-21AA-4F67-A14D-110CA1B1E11B}"/>
@@ -1261,12 +1298,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="52.453125" customWidth="1"/>
+    <col min="2" max="2" width="52.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="14.5">
+    <row r="1" spans="1:2" ht="14.4">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -1274,7 +1311,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="14.5">
+    <row r="2" spans="1:2" ht="14.4">
       <c r="A2" t="s">
         <v>29</v>
       </c>
@@ -1282,7 +1319,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="14.5">
+    <row r="3" spans="1:2" ht="14.4">
       <c r="A3" t="s">
         <v>31</v>
       </c>
@@ -1290,7 +1327,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="14.5">
+    <row r="4" spans="1:2" ht="14.4">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -1298,7 +1335,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="14.5">
+    <row r="5" spans="1:2" ht="14.4">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -1306,7 +1343,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="14.5">
+    <row r="6" spans="1:2" ht="14.4">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -1314,7 +1351,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="14.5">
+    <row r="7" spans="1:2" ht="14.4">
       <c r="A7" t="s">
         <v>31</v>
       </c>
@@ -1322,7 +1359,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="14.5">
+    <row r="8" spans="1:2" ht="14.4">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -1330,7 +1367,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="14.5">
+    <row r="9" spans="1:2" ht="14.4">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -1351,17 +1388,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.26953125" customWidth="1"/>
-    <col min="2" max="2" width="47.26953125" customWidth="1"/>
-    <col min="3" max="3" width="26.08984375" customWidth="1"/>
-    <col min="4" max="4" width="79.7265625" customWidth="1"/>
-    <col min="5" max="5" width="37.36328125" customWidth="1"/>
-    <col min="6" max="6" width="34.26953125" customWidth="1"/>
+    <col min="1" max="1" width="27.21875" customWidth="1"/>
+    <col min="2" max="2" width="47.21875" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" customWidth="1"/>
+    <col min="4" max="4" width="79.77734375" customWidth="1"/>
+    <col min="5" max="5" width="37.33203125" customWidth="1"/>
+    <col min="6" max="6" width="34.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.5">
+    <row r="1" spans="1:6" ht="14.4">
       <c r="A1" t="s">
         <v>33</v>
       </c>
@@ -1401,7 +1438,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="80.650000000000006" customHeight="1">
+    <row r="3" spans="1:6" ht="80.7" customHeight="1">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -1421,7 +1458,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="223.25" customHeight="1">
+    <row r="4" spans="1:6" ht="223.2" customHeight="1">
       <c r="A4" t="s">
         <v>47</v>
       </c>
@@ -1441,7 +1478,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="72.5" customHeight="1">
+    <row r="5" spans="1:6" ht="72.45" customHeight="1">
       <c r="A5" t="s">
         <v>47</v>
       </c>
@@ -1481,7 +1518,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="71" customHeight="1">
+    <row r="7" spans="1:6" ht="70.95" customHeight="1">
       <c r="A7" t="s">
         <v>53</v>
       </c>
@@ -1521,7 +1558,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="63.4" customHeight="1">
+    <row r="9" spans="1:6" ht="63.45" customHeight="1">
       <c r="A9" t="s">
         <v>59</v>
       </c>
@@ -1553,9 +1590,59 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{519B4DA3-55A1-4F7A-A01F-E188EB573246}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <sheetData/>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="46.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15">
+      <c r="A2" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="6"/>
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" spans="1:4" ht="15">
+      <c r="A3" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="D5" s="3"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1563,14 +1650,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="30.453125" customWidth="1"/>
-    <col min="2" max="2" width="16.08984375" customWidth="1"/>
+    <col min="1" max="1" width="30.44140625" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" customWidth="1"/>
     <col min="3" max="3" width="56" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="14.5">
+    <row r="1" spans="1:3" ht="14.4">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -1581,7 +1668,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="14.5">
+    <row r="2" spans="1:3" ht="14.4">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -1592,7 +1679,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="14.5">
+    <row r="3" spans="1:3" ht="14.4">
       <c r="A3" t="s">
         <v>68</v>
       </c>
@@ -1603,7 +1690,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="14.5">
+    <row r="4" spans="1:3" ht="14.4">
       <c r="A4" t="s">
         <v>69</v>
       </c>
@@ -1614,7 +1701,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="14.5">
+    <row r="5" spans="1:3" ht="14.4">
       <c r="A5" t="s">
         <v>69</v>
       </c>
@@ -1625,7 +1712,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="14.5">
+    <row r="6" spans="1:3" ht="14.4">
       <c r="A6" t="s">
         <v>70</v>
       </c>
@@ -1636,7 +1723,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="14.5">
+    <row r="7" spans="1:3" ht="14.4">
       <c r="A7" t="s">
         <v>70</v>
       </c>
@@ -1647,7 +1734,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="14.5">
+    <row r="8" spans="1:3" ht="14.4">
       <c r="A8" t="s">
         <v>71</v>
       </c>
@@ -1658,7 +1745,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="14.5">
+    <row r="9" spans="1:3" ht="14.4">
       <c r="A9" t="s">
         <v>71</v>
       </c>
@@ -1669,7 +1756,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="14.5">
+    <row r="10" spans="1:3" ht="14.4">
       <c r="A10" t="s">
         <v>72</v>
       </c>
@@ -1680,7 +1767,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="14.5">
+    <row r="11" spans="1:3" ht="14.4">
       <c r="A11" t="s">
         <v>72</v>
       </c>
@@ -1691,7 +1778,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="14.5">
+    <row r="12" spans="1:3" ht="14.4">
       <c r="A12" t="s">
         <v>73</v>
       </c>
@@ -1702,7 +1789,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="14.5">
+    <row r="13" spans="1:3" ht="14.4">
       <c r="A13" t="s">
         <v>73</v>
       </c>
@@ -1713,7 +1800,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="14.5">
+    <row r="14" spans="1:3" ht="14.4">
       <c r="A14" t="s">
         <v>74</v>
       </c>
@@ -1724,7 +1811,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="14.5">
+    <row r="15" spans="1:3" ht="14.4">
       <c r="A15" t="s">
         <v>74</v>
       </c>
@@ -1748,13 +1835,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="29.26953125" customWidth="1"/>
-    <col min="2" max="2" width="51.453125" customWidth="1"/>
+    <col min="1" max="1" width="29.21875" customWidth="1"/>
+    <col min="2" max="2" width="51.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="14.5">
+    <row r="1" spans="1:2" ht="14.4">
       <c r="A1" t="s">
         <v>33</v>
       </c>
@@ -1762,7 +1849,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="14.5">
+    <row r="2" spans="1:2" ht="14.4">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -1770,7 +1857,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="14.5">
+    <row r="3" spans="1:2" ht="14.4">
       <c r="A3" t="s">
         <v>69</v>
       </c>
@@ -1778,7 +1865,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="14.5">
+    <row r="4" spans="1:2" ht="14.4">
       <c r="A4" t="s">
         <v>70</v>
       </c>
@@ -1786,7 +1873,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="14.5">
+    <row r="5" spans="1:2" ht="14.4">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -1794,7 +1881,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="14.5">
+    <row r="6" spans="1:2" ht="14.4">
       <c r="A6" t="s">
         <v>72</v>
       </c>
@@ -1802,7 +1889,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="14.5">
+    <row r="7" spans="1:2" ht="14.4">
       <c r="A7" t="s">
         <v>73</v>
       </c>
@@ -1810,7 +1897,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="14.5">
+    <row r="8" spans="1:2" ht="14.4">
       <c r="A8" t="s">
         <v>74</v>
       </c>

</xml_diff>